<commit_message>
added a new dialogue system
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB9F7ED-0D7D-4CC2-A1E4-09522CD89ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A35982-8265-441E-963A-ED652C2938CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -994,12 +994,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1053,7 +1060,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1065,6 +1072,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1616,7 +1624,7 @@
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="7" t="s">
         <v>43</v>
       </c>
       <c r="J4" t="s">

</xml_diff>

<commit_message>
added add relics for debugging
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25445DB6-07B5-4749-ACC2-57EB25569AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7F6C2F-AB49-4852-AAEA-8DE1AED9A0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Revert "Merge remote-tracking branch 'origin/Scripting' into VTB3"
This reverts commit bccdddeb977198d3aad87af4250a77bf4e563238, reversing
changes made to f5731f7502f3839c649bb085ed4823ef59edc927.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Cards.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7F6C2F-AB49-4852-AAEA-8DE1AED9A0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25445DB6-07B5-4749-ACC2-57EB25569AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>

</xml_diff>